<commit_message>
Final UI with post processing
</commit_message>
<xml_diff>
--- a/input/parameters.xlsx
+++ b/input/parameters.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="86">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -136,7 +136,7 @@
     <t xml:space="preserve">executable</t>
   </si>
   <si>
-    <t xml:space="preserve">asteroid</t>
+    <t xml:space="preserve">landslide</t>
   </si>
   <si>
     <t xml:space="preserve">This is the executable file name which is run for the landslide simulation.</t>
@@ -250,13 +250,25 @@
     <t xml:space="preserve"> The time step for the YORP calculation in years</t>
   </si>
   <si>
+    <t xml:space="preserve">Nature</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Increasing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Increasing, Decreasing, Both</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Do you want YORP to be of specific kind? NEAs are spinning up.</t>
+  </si>
+  <si>
     <t xml:space="preserve">stoc_yorp</t>
   </si>
   <si>
     <t xml:space="preserve">No</t>
   </si>
   <si>
-    <t xml:space="preserve">Do you want yorp to be stochastic</t>
+    <t xml:space="preserve">Do you want yorp to be stochastic?</t>
   </si>
   <si>
     <t xml:space="preserve">Cummulative distribution</t>
@@ -275,9 +287,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="dd/mm/yy\ hh:mm"/>
+    <numFmt numFmtId="166" formatCode="0.00E+00"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -365,7 +378,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -383,6 +396,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -485,7 +502,7 @@
       </c>
       <c r="C5" s="4" t="n">
         <f aca="true">NOW()</f>
-        <v>45459.7230639566</v>
+        <v>45479.9232371508</v>
       </c>
       <c r="D5" s="3"/>
       <c r="E5" s="3" t="s">
@@ -499,7 +516,7 @@
       <c r="B6" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="3" t="n">
+      <c r="C6" s="5" t="n">
         <v>100000</v>
       </c>
       <c r="D6" s="3"/>
@@ -515,7 +532,7 @@
         <v>6</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="D7" s="3"/>
       <c r="E7" s="3" t="s">
@@ -786,7 +803,7 @@
         <v>6</v>
       </c>
       <c r="C13" s="3" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="D13" s="3"/>
       <c r="E13" s="3" t="s">
@@ -826,7 +843,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" zeroHeight="true" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20"/>
@@ -924,7 +941,7 @@
         <v>6</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>135</v>
+        <v>180</v>
       </c>
       <c r="D6" s="3"/>
       <c r="E6" s="3" t="s">
@@ -966,14 +983,31 @@
         <v>75</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="D9" s="3"/>
+      <c r="D9" s="3" t="s">
+        <v>77</v>
+      </c>
       <c r="E9" s="3" t="s">
-        <v>77</v>
+        <v>78</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3" t="s">
+        <v>81</v>
       </c>
     </row>
   </sheetData>
@@ -1022,19 +1056,19 @@
     </row>
     <row r="2" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>13</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Again commmiting because of last error
</commit_message>
<xml_diff>
--- a/input/parameters.xlsx
+++ b/input/parameters.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="General simulation parameters" sheetId="1" state="visible" r:id="rId2"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="99">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -55,10 +55,10 @@
     <t xml:space="preserve">The density of the asteroid</t>
   </si>
   <si>
-    <t xml:space="preserve">Angular velocity</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The non-dimensional angular velocity of the asteroid</t>
+    <t xml:space="preserve">Rotation period</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The initial time period of the rotation</t>
   </si>
   <si>
     <t xml:space="preserve">Output folder</t>
@@ -127,12 +127,27 @@
     <t xml:space="preserve">The timesteps after which the output of the landslide to be stored in the file. The location of output will be avialable in the parameter file under option verbose_dir. The option is valid only when verbose is selected</t>
   </si>
   <si>
+    <t xml:space="preserve">Landslide model</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Explicit-implicit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">explicit, explicit-implicit</t>
+  </si>
+  <si>
     <t xml:space="preserve">epsilon</t>
   </si>
   <si>
     <t xml:space="preserve">The non-dimensional height of the failed layer of the regolith. It should be smaller than Gamma and &lt;&lt;1</t>
   </si>
   <si>
+    <t xml:space="preserve">Minimum epsilon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maximum epsilon</t>
+  </si>
+  <si>
     <t xml:space="preserve">executable</t>
   </si>
   <si>
@@ -169,10 +184,13 @@
     <t xml:space="preserve">verbose</t>
   </si>
   <si>
+    <t xml:space="preserve">No</t>
+  </si>
+  <si>
     <t xml:space="preserve"> If you want to see the detailed simulation of landslides </t>
   </si>
   <si>
-    <t xml:space="preserve">Profile</t>
+    <t xml:space="preserve">Failure profile</t>
   </si>
   <si>
     <t xml:space="preserve">Uniform</t>
@@ -184,6 +202,18 @@
     <t xml:space="preserve">The profile of the failed regolith layer</t>
   </si>
   <si>
+    <t xml:space="preserve">Failure depth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Energy dependent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Constant, Energy dependent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The failure thickness is constant or does it vary with the impactor properties</t>
+  </si>
+  <si>
     <t xml:space="preserve">Landslide simulation period</t>
   </si>
   <si>
@@ -253,7 +283,7 @@
     <t xml:space="preserve">Nature</t>
   </si>
   <si>
-    <t xml:space="preserve">Increasing</t>
+    <t xml:space="preserve">Both</t>
   </si>
   <si>
     <t xml:space="preserve">Increasing, Decreasing, Both</t>
@@ -265,10 +295,19 @@
     <t xml:space="preserve">stoc_yorp</t>
   </si>
   <si>
-    <t xml:space="preserve">No</t>
-  </si>
-  <si>
     <t xml:space="preserve">Do you want yorp to be stochastic?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Explicit cutoff</t>
+  </si>
+  <si>
+    <t xml:space="preserve">To decide wether the impactor is explicit or implicit type. The explicit impactor will be greater than explict cutoff X diameter for catastrophic collisions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Implicit cutoff</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Impactors below implicit cutoff  X explicit cutoff X diameter for catastrophic collisions will be neglected</t>
   </si>
   <si>
     <t xml:space="preserve">Cummulative distribution</t>
@@ -486,7 +525,7 @@
         <v>6</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>0.7</v>
+        <v>4</v>
       </c>
       <c r="D4" s="3"/>
       <c r="E4" s="3" t="s">
@@ -502,7 +541,7 @@
       </c>
       <c r="C5" s="4" t="n">
         <f aca="true">NOW()</f>
-        <v>45479.9232371508</v>
+        <v>45486.4570787732</v>
       </c>
       <c r="D5" s="3"/>
       <c r="E5" s="3" t="s">
@@ -517,7 +556,7 @@
         <v>6</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>100000</v>
+        <v>2000000</v>
       </c>
       <c r="D6" s="3"/>
       <c r="E6" s="3" t="s">
@@ -532,7 +571,7 @@
         <v>6</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="D7" s="3"/>
       <c r="E7" s="3" t="s">
@@ -600,7 +639,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" zeroHeight="true" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20"/>
@@ -678,25 +717,25 @@
         <v>34</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C5" s="3" t="n">
-        <v>0.002</v>
-      </c>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>35</v>
       </c>
+      <c r="D5" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="E5" s="3"/>
     </row>
     <row r="6" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>37</v>
+        <v>6</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>0.002</v>
       </c>
       <c r="D6" s="3"/>
       <c r="E6" s="3" t="s">
@@ -711,120 +750,178 @@
         <v>6</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>0.01</v>
+        <v>0.001</v>
       </c>
       <c r="D7" s="3"/>
-      <c r="E7" s="3" t="s">
-        <v>40</v>
-      </c>
+      <c r="E7" s="3"/>
     </row>
     <row r="8" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>32</v>
+        <v>6</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>500</v>
+        <v>0.02</v>
       </c>
       <c r="D8" s="3"/>
-      <c r="E8" s="3" t="s">
-        <v>42</v>
-      </c>
+      <c r="E8" s="3"/>
     </row>
     <row r="9" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C9" s="3" t="n">
-        <v>1</v>
+        <v>13</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>42</v>
       </c>
       <c r="D9" s="3"/>
       <c r="E9" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>6</v>
       </c>
       <c r="C10" s="3" t="n">
-        <v>0.5</v>
+        <v>0.01</v>
       </c>
       <c r="D10" s="3"/>
       <c r="E10" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>21</v>
+        <v>32</v>
+      </c>
+      <c r="C11" s="3" t="n">
+        <v>500</v>
       </c>
       <c r="D11" s="3"/>
       <c r="E11" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3" t="s">
         <v>49</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>6</v>
       </c>
       <c r="C13" s="3" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="D13" s="3"/>
       <c r="E13" s="3" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B15" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="C15" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="D14" s="3" t="s">
+      <c r="D15" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="E14" s="3" t="s">
+      <c r="E15" s="3" t="s">
         <v>58</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C17" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="D17" s="3"/>
+      <c r="E17" s="3" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>68</v>
       </c>
     </row>
   </sheetData>
@@ -843,7 +940,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E1048576"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" zeroHeight="true" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20"/>
@@ -873,7 +970,7 @@
     </row>
     <row r="2" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>59</v>
+        <v>69</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>6</v>
@@ -883,29 +980,29 @@
       </c>
       <c r="D2" s="3"/>
       <c r="E2" s="3" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>61</v>
+        <v>71</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>13</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>62</v>
+        <v>72</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>63</v>
+        <v>73</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>6</v>
@@ -915,12 +1012,12 @@
       </c>
       <c r="D4" s="3"/>
       <c r="E4" s="3" t="s">
-        <v>66</v>
+        <v>76</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>67</v>
+        <v>77</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>6</v>
@@ -930,12 +1027,12 @@
       </c>
       <c r="D5" s="3"/>
       <c r="E5" s="3" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>6</v>
@@ -945,12 +1042,12 @@
       </c>
       <c r="D6" s="3"/>
       <c r="E6" s="3" t="s">
-        <v>70</v>
+        <v>80</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>6</v>
@@ -960,12 +1057,12 @@
       </c>
       <c r="D7" s="3"/>
       <c r="E7" s="3" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>6</v>
@@ -975,41 +1072,42 @@
       </c>
       <c r="D8" s="3"/>
       <c r="E8" s="3" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>13</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>20</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>80</v>
+        <v>21</v>
       </c>
       <c r="D10" s="3"/>
       <c r="E10" s="3" t="s">
-        <v>81</v>
-      </c>
-    </row>
+        <v>90</v>
+      </c>
+    </row>
+    <row r="1048576" customFormat="false" ht="60.4" hidden="true" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1026,7 +1124,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:AMJ1048576"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" zeroHeight="true" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20"/>
@@ -1056,21 +1154,56 @@
     </row>
     <row r="2" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>82</v>
+        <v>91</v>
       </c>
       <c r="B2" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="AMJ3" s="0"/>
+    </row>
+    <row r="4" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>85</v>
-      </c>
-    </row>
+      <c r="C4" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="1048573" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048574" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Updated regolith failure crietria  and seismic shaking
</commit_message>
<xml_diff>
--- a/input/parameters.xlsx
+++ b/input/parameters.xlsx
@@ -5,13 +5,13 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
-    <sheet name="General simulation parameters" sheetId="1" state="visible" r:id="rId2"/>
-    <sheet name="Landslide" sheetId="2" state="visible" r:id="rId3"/>
-    <sheet name="YORP" sheetId="3" state="visible" r:id="rId4"/>
-    <sheet name="Collision" sheetId="4" state="visible" r:id="rId5"/>
+    <sheet name="General simulation parameters" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Landslide" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="YORP" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Collision" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="114">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -112,6 +112,15 @@
     <t xml:space="preserve">It is the non-dimensional scale of the topography. Keep it smaller than 1.</t>
   </si>
   <si>
+    <t xml:space="preserve">Shallowness</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Variable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fixed, variable</t>
+  </si>
+  <si>
     <t xml:space="preserve">Friction angle</t>
   </si>
   <si>
@@ -127,18 +136,12 @@
     <t xml:space="preserve">The timesteps after which the output of the landslide to be stored in the file. The location of output will be avialable in the parameter file under option verbose_dir. The option is valid only when verbose is selected</t>
   </si>
   <si>
-    <t xml:space="preserve">Landslide model</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Explicit-implicit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">explicit, explicit-implicit</t>
-  </si>
-  <si>
     <t xml:space="preserve">epsilon</t>
   </si>
   <si>
+    <t xml:space="preserve">floar</t>
+  </si>
+  <si>
     <t xml:space="preserve">The non-dimensional height of the failed layer of the regolith. It should be smaller than Gamma and &lt;&lt;1</t>
   </si>
   <si>
@@ -220,6 +223,24 @@
     <t xml:space="preserve"> The simulation period after which the landslide will stop. This is the highest time for which landslide will be simulated</t>
   </si>
   <si>
+    <t xml:space="preserve">Seismic efficiency</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The seismic efficiency factor used in calculating sesmic energy in the body after impact</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cohesion constant</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Constant cohesion of the regolith</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cohesion linear</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Linear increase in the cohesion with depth</t>
+  </si>
+  <si>
     <t xml:space="preserve">Friction type</t>
   </si>
   <si>
@@ -301,13 +322,37 @@
     <t xml:space="preserve">Explicit cutoff</t>
   </si>
   <si>
-    <t xml:space="preserve">To decide wether the impactor is explicit or implicit type. The explicit impactor will be greater than explict cutoff X diameter for catastrophic collisions</t>
+    <t xml:space="preserve">To decide wether the impactor is explicit or implicit type. The explicit impactor will be greater than (explict cutoff ) X (diameter for catastrophic collisions)</t>
   </si>
   <si>
     <t xml:space="preserve">Implicit cutoff</t>
   </si>
   <si>
-    <t xml:space="preserve">Impactors below implicit cutoff  X explicit cutoff X diameter for catastrophic collisions will be neglected</t>
+    <t xml:space="preserve">Impactors below (implicit cutoff)  X (explicit cutoff) X (diameter for catastrophic collisions) will be neglected</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Impactor velocity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The impactor velocity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P wave speed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The P wave speed in the regolith as measured on the moon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Seismic quality factor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frequency</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Seismic frequency</t>
   </si>
   <si>
     <t xml:space="preserve">Cummulative distribution</t>
@@ -422,23 +467,23 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -454,8 +499,114 @@
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office">
+  <a:themeElements>
+    <a:clrScheme name="LibreOffice">
+      <a:dk1>
+        <a:srgbClr val="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:srgbClr val="ffffff"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="000000"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="ffffff"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="18a303"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="0369a3"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="a33e03"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8e03a3"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="c99c00"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="c9211e"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000ee"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="551a8b"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme>
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
@@ -468,6 +619,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="30"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="60"/>
     <col collapsed="false" customWidth="false" hidden="true" outlineLevel="0" max="1024" min="6" style="1" width="8.54"/>
+    <col collapsed="false" customWidth="false" hidden="true" outlineLevel="0" max="16384" min="1025" style="0" width="8.54"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -525,7 +677,7 @@
         <v>6</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D4" s="3"/>
       <c r="E4" s="3" t="s">
@@ -541,7 +693,7 @@
       </c>
       <c r="C5" s="4" t="n">
         <f aca="true">NOW()</f>
-        <v>45486.4570787732</v>
+        <v>45717.6574811063</v>
       </c>
       <c r="D5" s="3"/>
       <c r="E5" s="3" t="s">
@@ -556,7 +708,7 @@
         <v>6</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>2000000</v>
+        <v>1000000</v>
       </c>
       <c r="D6" s="3"/>
       <c r="E6" s="3" t="s">
@@ -635,11 +787,11 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E1048576"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" zeroHeight="true" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20"/>
@@ -648,6 +800,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="30"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="60"/>
     <col collapsed="false" customWidth="false" hidden="true" outlineLevel="0" max="1024" min="6" style="1" width="8.54"/>
+    <col collapsed="false" customWidth="false" hidden="true" outlineLevel="0" max="16384" min="1025" style="0" width="8.54"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -675,7 +828,7 @@
         <v>6</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>0.1</v>
+        <v>0.01</v>
       </c>
       <c r="D2" s="3"/>
       <c r="E2" s="3" t="s">
@@ -687,25 +840,25 @@
         <v>29</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" s="3" t="n">
-        <v>15</v>
-      </c>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>30</v>
       </c>
+      <c r="D3" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="E3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>32</v>
+        <v>6</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>200</v>
+        <v>35</v>
       </c>
       <c r="D4" s="3"/>
       <c r="E4" s="3" t="s">
@@ -717,47 +870,47 @@
         <v>34</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="C5" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="E5" s="3"/>
     </row>
     <row r="6" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
         <v>37</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>6</v>
+        <v>38</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="D6" s="3"/>
       <c r="E6" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>6</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>0.001</v>
+        <v>0.0001</v>
       </c>
       <c r="D7" s="3"/>
       <c r="E7" s="3"/>
     </row>
     <row r="8" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>6</v>
@@ -770,22 +923,22 @@
     </row>
     <row r="9" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>13</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D9" s="3"/>
       <c r="E9" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>6</v>
@@ -795,27 +948,27 @@
       </c>
       <c r="D10" s="3"/>
       <c r="E10" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C11" s="3" t="n">
         <v>500</v>
       </c>
       <c r="D11" s="3"/>
       <c r="E11" s="3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>6</v>
@@ -825,12 +978,12 @@
       </c>
       <c r="D12" s="3"/>
       <c r="E12" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>6</v>
@@ -840,90 +993,136 @@
       </c>
       <c r="D13" s="3"/>
       <c r="E13" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>20</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D14" s="3"/>
       <c r="E14" s="3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>13</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>13</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>6</v>
       </c>
       <c r="C17" s="3" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="D17" s="3"/>
       <c r="E17" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B18" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C18" s="5" t="n">
+        <v>1E-006</v>
+      </c>
+      <c r="D18" s="3"/>
+      <c r="E18" s="3" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C19" s="5" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D19" s="3"/>
+      <c r="E19" s="3" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C20" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="3"/>
+      <c r="E20" s="3" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B21" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C18" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="D18" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="E18" s="3" t="s">
-        <v>68</v>
-      </c>
-    </row>
+      <c r="C21" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -936,7 +1135,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
@@ -949,6 +1148,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="30"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="60"/>
     <col collapsed="false" customWidth="false" hidden="true" outlineLevel="0" max="1024" min="6" style="1" width="8.54"/>
+    <col collapsed="false" customWidth="false" hidden="true" outlineLevel="0" max="16384" min="1025" style="0" width="8.54"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -970,7 +1170,7 @@
     </row>
     <row r="2" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>6</v>
@@ -980,29 +1180,29 @@
       </c>
       <c r="D2" s="3"/>
       <c r="E2" s="3" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>13</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>6</v>
@@ -1012,12 +1212,12 @@
       </c>
       <c r="D4" s="3"/>
       <c r="E4" s="3" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>6</v>
@@ -1027,12 +1227,12 @@
       </c>
       <c r="D5" s="3"/>
       <c r="E5" s="3" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>6</v>
@@ -1042,12 +1242,12 @@
       </c>
       <c r="D6" s="3"/>
       <c r="E6" s="3" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>6</v>
@@ -1057,12 +1257,12 @@
       </c>
       <c r="D7" s="3"/>
       <c r="E7" s="3" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>6</v>
@@ -1072,29 +1272,29 @@
       </c>
       <c r="D8" s="3"/>
       <c r="E8" s="3" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>13</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>20</v>
@@ -1104,7 +1304,7 @@
       </c>
       <c r="D10" s="3"/>
       <c r="E10" s="3" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
     </row>
     <row r="1048576" customFormat="false" ht="60.4" hidden="true" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -1120,22 +1320,22 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AMJ1048576"/>
-  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" zeroHeight="true" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:E9"/>
+  <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="12.8" zeroHeight="true" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="60"/>
-    <col collapsed="false" customWidth="false" hidden="true" outlineLevel="0" max="1024" min="6" style="1" width="8.54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="17.77"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12.74"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="18.99"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="79.41"/>
+    <col collapsed="false" customWidth="false" hidden="true" outlineLevel="0" max="16384" min="6" style="0" width="10.16"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1152,24 +1352,24 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="70.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>6</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="D2" s="3"/>
       <c r="E2" s="3" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="70.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>6</v>
@@ -1179,38 +1379,108 @@
       </c>
       <c r="D3" s="3"/>
       <c r="E3" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="AMJ3" s="0"/>
-    </row>
-    <row r="4" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="62.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>95</v>
+        <v>66</v>
       </c>
       <c r="B4" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="5" t="n">
+        <v>1E-005</v>
+      </c>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>5500</v>
+      </c>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="81.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="81.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>1500</v>
+      </c>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="81.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C8" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="71.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="1048573" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048574" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048575" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048576" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false"/>
+      <c r="C9" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>113</v>
+      </c>
+    </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Implemented recent suggestions. Debugged for errors
</commit_message>
<xml_diff>
--- a/input/parameters.xlsx
+++ b/input/parameters.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="General simulation parameters" sheetId="1" state="visible" r:id="rId3"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="112">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -187,9 +187,6 @@
     <t xml:space="preserve">verbose</t>
   </si>
   <si>
-    <t xml:space="preserve">No</t>
-  </si>
-  <si>
     <t xml:space="preserve"> If you want to see the detailed simulation of landslides </t>
   </si>
   <si>
@@ -223,112 +220,109 @@
     <t xml:space="preserve"> The simulation period after which the landslide will stop. This is the highest time for which landslide will be simulated</t>
   </si>
   <si>
+    <t xml:space="preserve">Cohesion constant</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Constant cohesion of the regolith</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cohesion linear</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Linear increase in the cohesion with depth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Friction type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Constant, Variable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">If you want a constant friction angle through out the lanslide, select constant otherwise choose variable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thermal inertia </t>
+  </si>
+  <si>
+    <t xml:space="preserve">atype</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C-Type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C-Type, S-Type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Typeof asteroid, C-Type or S-Type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c_YORP</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> For calculating YORP torques</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c_reor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">To calulate the probability of collisional reoriention after at very slow spin rate </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Obliquity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The obliquity of the asteroid </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Semi major axis</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> The semi major axis of the asteroid</t>
+  </si>
+  <si>
+    <t xml:space="preserve">h_yorp</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> The time step for the YORP calculation in years</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nature</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Both</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Increasing, Decreasing, Both</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Do you want YORP to be of specific kind? NEAs are spinning up.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stoc_yorp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Do you want yorp to be stochastic?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Explicit cutoff</t>
+  </si>
+  <si>
+    <t xml:space="preserve">To decide wether the impactor is explicit or implicit type. The explicit impactor will be greater than (explict cutoff ) X (diameter for catastrophic collisions)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Implicit cutoff</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Impactors below (implicit cutoff)  X (explicit cutoff) X (diameter for catastrophic collisions) will be neglected</t>
+  </si>
+  <si>
     <t xml:space="preserve">Seismic efficiency</t>
   </si>
   <si>
     <t xml:space="preserve">The seismic efficiency factor used in calculating sesmic energy in the body after impact</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cohesion constant</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Constant cohesion of the regolith</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cohesion linear</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Linear increase in the cohesion with depth</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Friction type</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Constant</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Constant, Variable</t>
-  </si>
-  <si>
-    <t xml:space="preserve">If you want a constant friction angle through out the lanslide, select constant otherwise choose variable</t>
-  </si>
-  <si>
-    <t xml:space="preserve">K</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thermal inertia </t>
-  </si>
-  <si>
-    <t xml:space="preserve">atype</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C-Type</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C-Type, S-Type</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Typeof asteroid, C-Type or S-Type</t>
-  </si>
-  <si>
-    <t xml:space="preserve">c_YORP</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> For calculating YORP torques</t>
-  </si>
-  <si>
-    <t xml:space="preserve">c_reor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">To calulate the probability of collisional reoriention after at very slow spin rate </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Obliquity</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The obliquity of the asteroid </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Semi major axis</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> The semi major axis of the asteroid</t>
-  </si>
-  <si>
-    <t xml:space="preserve">h_yorp</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> The time step for the YORP calculation in years</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nature</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Both</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Increasing, Decreasing, Both</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Do you want YORP to be of specific kind? NEAs are spinning up.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">stoc_yorp</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Do you want yorp to be stochastic?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Explicit cutoff</t>
-  </si>
-  <si>
-    <t xml:space="preserve">To decide wether the impactor is explicit or implicit type. The explicit impactor will be greater than (explict cutoff ) X (diameter for catastrophic collisions)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Implicit cutoff</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Impactors below (implicit cutoff)  X (explicit cutoff) X (diameter for catastrophic collisions) will be neglected</t>
   </si>
   <si>
     <t xml:space="preserve">Impactor velocity</t>
@@ -618,8 +612,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="20"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="30"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="60"/>
-    <col collapsed="false" customWidth="false" hidden="true" outlineLevel="0" max="1024" min="6" style="1" width="8.54"/>
-    <col collapsed="false" customWidth="false" hidden="true" outlineLevel="0" max="16384" min="1025" style="0" width="8.54"/>
+    <col collapsed="false" customWidth="false" hidden="true" outlineLevel="0" max="16384" min="6" style="1" width="8.54"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -677,7 +670,7 @@
         <v>6</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D4" s="3"/>
       <c r="E4" s="3" t="s">
@@ -693,7 +686,7 @@
       </c>
       <c r="C5" s="4" t="n">
         <f aca="true">NOW()</f>
-        <v>45717.6574811063</v>
+        <v>45731.6289003361</v>
       </c>
       <c r="D5" s="3"/>
       <c r="E5" s="3" t="s">
@@ -708,7 +701,7 @@
         <v>6</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>1000000</v>
+        <v>100000</v>
       </c>
       <c r="D6" s="3"/>
       <c r="E6" s="3" t="s">
@@ -723,7 +716,7 @@
         <v>6</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="D7" s="3"/>
       <c r="E7" s="3" t="s">
@@ -799,8 +792,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="20"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="30"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="60"/>
-    <col collapsed="false" customWidth="false" hidden="true" outlineLevel="0" max="1024" min="6" style="1" width="8.54"/>
-    <col collapsed="false" customWidth="false" hidden="true" outlineLevel="0" max="16384" min="1025" style="0" width="8.54"/>
+    <col collapsed="false" customWidth="false" hidden="true" outlineLevel="0" max="16384" min="6" style="1" width="8.54"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -873,7 +865,7 @@
         <v>35</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>200</v>
+        <v>50</v>
       </c>
       <c r="D5" s="3"/>
       <c r="E5" s="3" t="s">
@@ -959,7 +951,7 @@
         <v>35</v>
       </c>
       <c r="C11" s="3" t="n">
-        <v>500</v>
+        <v>2000</v>
       </c>
       <c r="D11" s="3"/>
       <c r="E11" s="3" t="s">
@@ -974,7 +966,7 @@
         <v>6</v>
       </c>
       <c r="C12" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D12" s="3"/>
       <c r="E12" s="3" t="s">
@@ -1004,124 +996,110 @@
         <v>20</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>54</v>
+        <v>21</v>
       </c>
       <c r="D14" s="3"/>
       <c r="E14" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>13</v>
       </c>
       <c r="C15" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D15" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="D15" s="3" t="s">
+      <c r="E15" s="3" t="s">
         <v>58</v>
-      </c>
-      <c r="E15" s="3" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>13</v>
       </c>
       <c r="C16" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="D16" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="D16" s="3" t="s">
+      <c r="E16" s="3" t="s">
         <v>62</v>
-      </c>
-      <c r="E16" s="3" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>6</v>
       </c>
       <c r="C17" s="3" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="D17" s="3"/>
       <c r="E17" s="3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>6</v>
       </c>
       <c r="C18" s="5" t="n">
-        <v>1E-006</v>
+        <v>0.1</v>
       </c>
       <c r="D18" s="3"/>
       <c r="E18" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>6</v>
       </c>
       <c r="C19" s="5" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="D19" s="3"/>
       <c r="E19" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D20" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="B20" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C20" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" s="3"/>
       <c r="E20" s="3" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="B21" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C21" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="D21" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="E21" s="3" t="s">
-        <v>75</v>
-      </c>
-    </row>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1147,8 +1125,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="20"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="30"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="60"/>
-    <col collapsed="false" customWidth="false" hidden="true" outlineLevel="0" max="1024" min="6" style="1" width="8.54"/>
-    <col collapsed="false" customWidth="false" hidden="true" outlineLevel="0" max="16384" min="1025" style="0" width="8.54"/>
+    <col collapsed="false" customWidth="false" hidden="true" outlineLevel="0" max="16384" min="6" style="1" width="8.54"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1170,7 +1147,7 @@
     </row>
     <row r="2" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>6</v>
@@ -1180,29 +1157,29 @@
       </c>
       <c r="D2" s="3"/>
       <c r="E2" s="3" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>13</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>6</v>
@@ -1212,12 +1189,12 @@
       </c>
       <c r="D4" s="3"/>
       <c r="E4" s="3" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>6</v>
@@ -1227,12 +1204,12 @@
       </c>
       <c r="D5" s="3"/>
       <c r="E5" s="3" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>6</v>
@@ -1242,12 +1219,12 @@
       </c>
       <c r="D6" s="3"/>
       <c r="E6" s="3" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>6</v>
@@ -1257,12 +1234,12 @@
       </c>
       <c r="D7" s="3"/>
       <c r="E7" s="3" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>6</v>
@@ -1272,29 +1249,29 @@
       </c>
       <c r="D8" s="3"/>
       <c r="E8" s="3" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>13</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>20</v>
@@ -1304,7 +1281,7 @@
       </c>
       <c r="D10" s="3"/>
       <c r="E10" s="3" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
     </row>
     <row r="1048576" customFormat="false" ht="60.4" hidden="true" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -1327,12 +1304,12 @@
   <dimension ref="A1:E9"/>
   <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="12.8" zeroHeight="true" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="17.77"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12.74"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="18.99"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="79.41"/>
-    <col collapsed="false" customWidth="false" hidden="true" outlineLevel="0" max="16384" min="6" style="0" width="10.16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="17.77"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="12.74"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="18.99"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="79.41"/>
+    <col collapsed="false" customWidth="false" hidden="true" outlineLevel="0" max="16384" min="6" style="1" width="10.16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1354,7 +1331,7 @@
     </row>
     <row r="2" customFormat="false" ht="70.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>6</v>
@@ -1364,12 +1341,12 @@
       </c>
       <c r="D2" s="3"/>
       <c r="E2" s="3" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="70.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>6</v>
@@ -1379,27 +1356,27 @@
       </c>
       <c r="D3" s="3"/>
       <c r="E3" s="3" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="62.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>66</v>
+        <v>98</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>6</v>
       </c>
       <c r="C4" s="5" t="n">
-        <v>1E-005</v>
+        <v>1E-006</v>
       </c>
       <c r="D4" s="3"/>
       <c r="E4" s="3" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>6</v>
@@ -1409,12 +1386,12 @@
       </c>
       <c r="D5" s="3"/>
       <c r="E5" s="3" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="81.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>6</v>
@@ -1424,12 +1401,12 @@
       </c>
       <c r="D6" s="3"/>
       <c r="E6" s="3" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="81.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>6</v>
@@ -1439,39 +1416,39 @@
       </c>
       <c r="D7" s="3"/>
       <c r="E7" s="3" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="81.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>6</v>
       </c>
       <c r="C8" s="5" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="D8" s="3"/>
       <c r="E8" s="3" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="71.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>13</v>
       </c>
       <c r="C9" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="E9" s="3" t="s">
         <v>111</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>113</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Generalized it to any axisymmetric case
</commit_message>
<xml_diff>
--- a/input/parameters.xlsx
+++ b/input/parameters.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="General simulation parameters" sheetId="1" state="visible" r:id="rId3"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="120">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -40,13 +40,28 @@
     <t xml:space="preserve">Help</t>
   </si>
   <si>
+    <t xml:space="preserve">Asteroid</t>
+  </si>
+  <si>
+    <t xml:space="preserve">str</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spherical</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bennu, Ryugu, Itokawa, Spherical</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The shape of real asteroids</t>
+  </si>
+  <si>
     <t xml:space="preserve">Diameter</t>
   </si>
   <si>
     <t xml:space="preserve">float</t>
   </si>
   <si>
-    <t xml:space="preserve">The diameter of the asteroid</t>
+    <t xml:space="preserve">The diameter of the asteroid. Used only when spherical is selected.</t>
   </si>
   <si>
     <t xml:space="preserve">Density</t>
@@ -64,10 +79,7 @@
     <t xml:space="preserve">Output folder</t>
   </si>
   <si>
-    <t xml:space="preserve">str</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Crater</t>
+    <t xml:space="preserve">Debug</t>
   </si>
   <si>
     <t xml:space="preserve">The output folder of the simulations</t>
@@ -88,66 +100,57 @@
     <t xml:space="preserve">Dimension</t>
   </si>
   <si>
+    <t xml:space="preserve">1D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1D, 2D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dimension of simulation 1D or 2D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Collision</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bool</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Do you want to include the effect of collision on spin rate?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Landslide</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Do you want to include the effect of landslide on spin rate and shape?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YORP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Do you want to include the effect of YORP on spin rate?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Friction angle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Friction angle of the regolith</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dump</t>
+  </si>
+  <si>
     <t xml:space="preserve">int</t>
   </si>
   <si>
-    <t xml:space="preserve">2D</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1D, 2D</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dimension of simulation 1D or 2D</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Collision</t>
-  </si>
-  <si>
-    <t xml:space="preserve">bool</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Yes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Do you want to include the effect of collision on spin rate?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Landslide</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Do you want to include the effect of lanslide on spin rate and shape?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">YORP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Do you want to include the effect of YORP on spin rate?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gamma</t>
-  </si>
-  <si>
-    <t xml:space="preserve">It is the non-dimensional scale of the topography. Keep it smaller than 1.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Friction angle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Friction angle of the regolith</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dump</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The timesteps after which the output of the landslide to be stored in the file. The location of output will be avialable in the parameter file under option verbose_dir. The option is valid only when verbose is selected</t>
+    <t xml:space="preserve">The time steps after which the output of the landslide to be stored in the file. The location of output will be available in the parameters file under the option verbose_dir. The option is valid only when verbose is selected</t>
   </si>
   <si>
     <t xml:space="preserve">epsilon</t>
   </si>
   <si>
-    <t xml:space="preserve">floar</t>
-  </si>
-  <si>
     <t xml:space="preserve">The non-dimensional height of the failed layer of the regolith. It should be smaller than Gamma and &lt;&lt;1</t>
   </si>
   <si>
@@ -190,13 +193,13 @@
     <t xml:space="preserve">Phi for the case of spherical</t>
   </si>
   <si>
-    <t xml:space="preserve">theta</t>
+    <t xml:space="preserve">Minmod Limiter</t>
   </si>
   <si>
     <t xml:space="preserve"> Top be used in the min-mod limiter</t>
   </si>
   <si>
-    <t xml:space="preserve">weight</t>
+    <t xml:space="preserve">Correction weight</t>
   </si>
   <si>
     <t xml:space="preserve"> To be used for the Runge-Kutta scheme</t>
@@ -253,7 +256,7 @@
     <t xml:space="preserve">C-Type, S-Type</t>
   </si>
   <si>
-    <t xml:space="preserve">Typeof asteroid, C-Type or S-Type</t>
+    <t xml:space="preserve">Type of asteroid, C-Type or S-Type</t>
   </si>
   <si>
     <t xml:space="preserve">c_YORP</t>
@@ -265,7 +268,7 @@
     <t xml:space="preserve">c_reor</t>
   </si>
   <si>
-    <t xml:space="preserve">To calulate the probability of collisional reoriention after at very slow spin rate </t>
+    <t xml:space="preserve">To calculate the probability of collisional reorientation after at very slow spin rate </t>
   </si>
   <si>
     <t xml:space="preserve">Obliquity</t>
@@ -289,7 +292,7 @@
     <t xml:space="preserve">Nature</t>
   </si>
   <si>
-    <t xml:space="preserve">Both</t>
+    <t xml:space="preserve">Increasing</t>
   </si>
   <si>
     <t xml:space="preserve">Increasing, Decreasing, Both</t>
@@ -301,13 +304,16 @@
     <t xml:space="preserve">stoc_yorp</t>
   </si>
   <si>
+    <t xml:space="preserve">No</t>
+  </si>
+  <si>
     <t xml:space="preserve">Do you want yorp to be stochastic?</t>
   </si>
   <si>
     <t xml:space="preserve">Explicit cutoff</t>
   </si>
   <si>
-    <t xml:space="preserve">To decide wether the impactor is explicit or implicit type. The explicit impactor will be greater than (explict cutoff ) X (diameter for catastrophic collisions)</t>
+    <t xml:space="preserve">To decide wether the impactor is explicit or implicit type. The explicit impactor will be greater than (explicit cutoff ) X (diameter for catastrophic collisions)</t>
   </si>
   <si>
     <t xml:space="preserve">Implicit cutoff</t>
@@ -319,19 +325,34 @@
     <t xml:space="preserve">Seismic efficiency</t>
   </si>
   <si>
-    <t xml:space="preserve">The seismic efficiency factor used in calculating sesmic energy in the body after impact</t>
+    <t xml:space="preserve">The seismic efficiency factor used in calculating seismic energy in the body after impact</t>
   </si>
   <si>
     <t xml:space="preserve">Impactor velocity</t>
   </si>
   <si>
-    <t xml:space="preserve">The impactor velocity</t>
+    <t xml:space="preserve">The average velocity of impactors</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Velocity file</t>
+  </si>
+  <si>
+    <t xml:space="preserve">vel_dist.txt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">File containing velocity distribution</t>
   </si>
   <si>
     <t xml:space="preserve">Impactor Crater ratio</t>
   </si>
   <si>
+    <t xml:space="preserve">Ratio of impactor to Crater diameter</t>
+  </si>
+  <si>
     <t xml:space="preserve">Depth to Diameter ratio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ratio of Crater depth to Diameter</t>
   </si>
   <si>
     <t xml:space="preserve">P wave speed</t>
@@ -459,7 +480,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -474,6 +495,10 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -607,7 +632,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" zeroHeight="true" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20"/>
@@ -642,149 +667,166 @@
       <c r="B2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="3" t="n">
-        <v>500</v>
-      </c>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3" t="s">
+      <c r="C2" s="3" t="s">
         <v>7</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>1250</v>
+        <v>500</v>
       </c>
       <c r="D3" s="3"/>
       <c r="E3" s="3" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>4</v>
+        <v>1250</v>
       </c>
       <c r="D4" s="3"/>
       <c r="E4" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>14</v>
+        <v>11</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>4.3</v>
       </c>
       <c r="D5" s="3"/>
       <c r="E5" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="5" t="n">
-        <v>0.1</v>
+      <c r="C6" s="5" t="s">
+        <v>18</v>
       </c>
       <c r="D6" s="3"/>
       <c r="E6" s="3" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C7" s="3" t="n">
-        <v>1</v>
+        <v>11</v>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>0.01</v>
       </c>
       <c r="D7" s="3"/>
       <c r="E7" s="3" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="D8" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3" t="s">
         <v>23</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="D9" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="E9" s="3" t="s">
         <v>27</v>
-      </c>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B10" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="B10" s="3" t="s">
-        <v>26</v>
-      </c>
       <c r="C10" s="3" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="D10" s="3"/>
       <c r="E10" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="D11" s="3"/>
       <c r="E11" s="3" t="s">
-        <v>32</v>
+        <v>33</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3" t="s">
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -833,272 +875,258 @@
     </row>
     <row r="2" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>0.01</v>
+        <v>35</v>
       </c>
       <c r="D2" s="3"/>
       <c r="E2" s="3" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>6</v>
+        <v>39</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>35</v>
+        <v>50</v>
       </c>
       <c r="D3" s="3"/>
       <c r="E3" s="3" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>30</v>
+        <v>0.01</v>
       </c>
       <c r="D4" s="3"/>
       <c r="E4" s="3" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>40</v>
+        <v>11</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>0.01</v>
+        <v>0.0001</v>
       </c>
       <c r="D5" s="3"/>
-      <c r="E5" s="3" t="s">
-        <v>41</v>
-      </c>
+      <c r="E5" s="3"/>
     </row>
     <row r="6" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>0.0001</v>
+        <v>0.02</v>
       </c>
       <c r="D6" s="3"/>
       <c r="E6" s="3"/>
     </row>
     <row r="7" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="3" t="n">
-        <v>0.02</v>
+      <c r="C7" s="3" t="s">
+        <v>46</v>
       </c>
       <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
+      <c r="E7" s="3" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>45</v>
+        <v>11</v>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="D8" s="3"/>
       <c r="E8" s="3" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>6</v>
+        <v>39</v>
       </c>
       <c r="C9" s="3" t="n">
-        <v>0.15</v>
+        <v>1000</v>
       </c>
       <c r="D9" s="3"/>
       <c r="E9" s="3" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="C10" s="3" t="n">
-        <v>1000</v>
+        <v>200</v>
       </c>
       <c r="D10" s="3"/>
       <c r="E10" s="3" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="C11" s="3" t="n">
         <v>200</v>
       </c>
       <c r="D11" s="3"/>
       <c r="E11" s="3" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="C12" s="3" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="D12" s="3"/>
       <c r="E12" s="3" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C13" s="3" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="D13" s="3"/>
       <c r="E13" s="3" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C14" s="3" t="n">
-        <v>0.5</v>
+        <v>29</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>30</v>
       </c>
       <c r="D14" s="3"/>
       <c r="E14" s="3" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>27</v>
+        <v>11</v>
+      </c>
+      <c r="C15" s="3" t="n">
+        <v>10</v>
       </c>
       <c r="D15" s="3"/>
       <c r="E15" s="3" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C16" s="3" t="n">
-        <v>2</v>
+        <v>11</v>
+      </c>
+      <c r="C16" s="6" t="n">
+        <v>0.1</v>
       </c>
       <c r="D16" s="3"/>
       <c r="E16" s="3" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C17" s="5" t="n">
-        <v>0.1</v>
+        <v>11</v>
+      </c>
+      <c r="C17" s="6" t="n">
+        <v>1</v>
       </c>
       <c r="D17" s="3"/>
       <c r="E17" s="3" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C18" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D18" s="3"/>
+      <c r="C18" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>70</v>
+      </c>
       <c r="E18" s="3" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C19" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="D19" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="E19" s="3" t="s">
-        <v>70</v>
-      </c>
-    </row>
+        <v>71</v>
+      </c>
+    </row>
+    <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -1148,141 +1176,141 @@
     </row>
     <row r="2" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C2" s="3" t="n">
         <v>0.01</v>
       </c>
       <c r="D2" s="3"/>
       <c r="E2" s="3" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>0.7</v>
+        <v>0.081</v>
       </c>
       <c r="D4" s="3"/>
       <c r="E4" s="3" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C5" s="3" t="n">
         <v>0.9</v>
       </c>
       <c r="D5" s="3"/>
       <c r="E5" s="3" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C6" s="3" t="n">
         <v>180</v>
       </c>
       <c r="D6" s="3"/>
       <c r="E6" s="3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C7" s="3" t="n">
         <v>2.3</v>
       </c>
       <c r="D7" s="3"/>
       <c r="E7" s="3" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C8" s="3" t="n">
         <v>50</v>
       </c>
       <c r="D8" s="3"/>
       <c r="E8" s="3" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>27</v>
+        <v>93</v>
       </c>
       <c r="D10" s="3"/>
       <c r="E10" s="3" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="1048576" customFormat="false" ht="60.4" hidden="true" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -1302,14 +1330,14 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
-  <sheetFormatPr defaultColWidth="10.16015625" defaultRowHeight="12.8" zeroHeight="true" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:E12"/>
+  <sheetFormatPr defaultColWidth="10.1640625" defaultRowHeight="12.8" zeroHeight="true" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="15.19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="17.83"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.86"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="12.74"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="18.99"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="79.41"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="79.42"/>
     <col collapsed="false" customWidth="false" hidden="true" outlineLevel="0" max="16384" min="6" style="1" width="10.16"/>
   </cols>
   <sheetData>
@@ -1332,150 +1360,169 @@
     </row>
     <row r="2" customFormat="false" ht="70.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C2" s="3" t="n">
         <v>0.1</v>
       </c>
       <c r="D2" s="3"/>
       <c r="E2" s="3" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="70.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C3" s="3" t="n">
         <v>0.1</v>
       </c>
       <c r="D3" s="3"/>
       <c r="E3" s="3" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="62.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C4" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="C4" s="6" t="n">
         <v>1E-006</v>
       </c>
       <c r="D4" s="3"/>
       <c r="E4" s="3" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="40.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="62.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C5" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="C5" s="6" t="n">
         <v>5500</v>
       </c>
       <c r="D5" s="3"/>
       <c r="E5" s="3" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="41.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="62.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="5" t="n">
+      <c r="C6" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="41.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7" s="6" t="n">
         <v>30</v>
       </c>
-      <c r="D6" s="3"/>
-      <c r="E6" s="3"/>
-    </row>
-    <row r="7" customFormat="false" ht="50.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C7" s="5" t="n">
+      <c r="D7" s="3"/>
+      <c r="E7" s="3" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="50.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" s="6" t="n">
         <v>0.2</v>
-      </c>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-    </row>
-    <row r="8" customFormat="false" ht="81.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C8" s="5" t="n">
-        <v>100</v>
       </c>
       <c r="D8" s="3"/>
       <c r="E8" s="3" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="81.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C9" s="5" t="n">
-        <v>1500</v>
+        <v>11</v>
+      </c>
+      <c r="C9" s="6" t="n">
+        <v>100</v>
       </c>
       <c r="D9" s="3"/>
       <c r="E9" s="3" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="81.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C10" s="5" t="n">
-        <v>1</v>
+        <v>11</v>
+      </c>
+      <c r="C10" s="6" t="n">
+        <v>1500</v>
       </c>
       <c r="D10" s="3"/>
       <c r="E10" s="3" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="71.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="81.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>111</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="C11" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="3"/>
       <c r="E11" s="3" t="s">
-        <v>112</v>
+        <v>115</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="71.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>119</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Complete axisymmetric details added
</commit_message>
<xml_diff>
--- a/input/parameters.xlsx
+++ b/input/parameters.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="General simulation parameters" sheetId="1" state="visible" r:id="rId3"/>
@@ -13,6 +13,9 @@
     <sheet name="YORP" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Collision" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
+  <definedNames>
+    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">YORP!$A$1048576</definedName>
+  </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
@@ -23,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="135">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -46,13 +49,13 @@
     <t xml:space="preserve">str</t>
   </si>
   <si>
-    <t xml:space="preserve">Spherical</t>
+    <t xml:space="preserve">Bennu</t>
   </si>
   <si>
     <t xml:space="preserve">Bennu, Ryugu, Itokawa, Spherical</t>
   </si>
   <si>
-    <t xml:space="preserve">The shape of real asteroids</t>
+    <t xml:space="preserve"> The initial shape of asteroid. Currently, the software includes shape for Oblate, Prolate, Spherical, Bennu, Regolith and Itokawa.</t>
   </si>
   <si>
     <t xml:space="preserve">Diameter</t>
@@ -79,7 +82,7 @@
     <t xml:space="preserve">Output folder</t>
   </si>
   <si>
-    <t xml:space="preserve">Debug</t>
+    <t xml:space="preserve">Spherical_1</t>
   </si>
   <si>
     <t xml:space="preserve">The output folder of the simulations</t>
@@ -100,7 +103,7 @@
     <t xml:space="preserve">Dimension</t>
   </si>
   <si>
-    <t xml:space="preserve">1D</t>
+    <t xml:space="preserve">2D</t>
   </si>
   <si>
     <t xml:space="preserve">1D, 2D</t>
@@ -133,12 +136,15 @@
     <t xml:space="preserve">Do you want to include the effect of YORP on spin rate?</t>
   </si>
   <si>
-    <t xml:space="preserve">Friction angle</t>
+    <t xml:space="preserve">Static Friction angle</t>
   </si>
   <si>
     <t xml:space="preserve">Friction angle of the regolith</t>
   </si>
   <si>
+    <t xml:space="preserve">Dynamic Friction angle</t>
+  </si>
+  <si>
     <t xml:space="preserve">dump</t>
   </si>
   <si>
@@ -169,6 +175,30 @@
     <t xml:space="preserve">This is the executable file name which is run for the landslide simulation.</t>
   </si>
   <si>
+    <t xml:space="preserve">Solver</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Runge-Kutta 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LXF first order, Predictor Corrector, Runge-Kutta 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The solver to be used for the integration</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reconstruction</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cartesian conserved variables</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Primitive variables, Conserved variables, Cartesian conserved variables</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The reconstruction scheme to be used for the higher order accuracy</t>
+  </si>
+  <si>
     <t xml:space="preserve">offset</t>
   </si>
   <si>
@@ -199,19 +229,13 @@
     <t xml:space="preserve"> Top be used in the min-mod limiter</t>
   </si>
   <si>
-    <t xml:space="preserve">Correction weight</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> To be used for the Runge-Kutta scheme</t>
-  </si>
-  <si>
     <t xml:space="preserve">verbose</t>
   </si>
   <si>
     <t xml:space="preserve"> If you want to see the detailed simulation of landslides </t>
   </si>
   <si>
-    <t xml:space="preserve">Landslide simulation period</t>
+    <t xml:space="preserve">Maximum simulation period</t>
   </si>
   <si>
     <t xml:space="preserve"> The simulation period after which the landslide will stop. This is the highest time for which landslide will be simulated</t>
@@ -232,7 +256,7 @@
     <t xml:space="preserve">Friction type</t>
   </si>
   <si>
-    <t xml:space="preserve">Variable</t>
+    <t xml:space="preserve">Constant</t>
   </si>
   <si>
     <t xml:space="preserve">Constant, Variable</t>
@@ -301,6 +325,12 @@
     <t xml:space="preserve">Do you want YORP to be of specific kind? NEAs are spinning up.</t>
   </si>
   <si>
+    <t xml:space="preserve">N_stoch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The number of landslides after which stochastic YORP resets</t>
+  </si>
+  <si>
     <t xml:space="preserve">stoc_yorp</t>
   </si>
   <si>
@@ -316,12 +346,6 @@
     <t xml:space="preserve">To decide wether the impactor is explicit or implicit type. The explicit impactor will be greater than (explicit cutoff ) X (diameter for catastrophic collisions)</t>
   </si>
   <si>
-    <t xml:space="preserve">Implicit cutoff</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Impactors below (implicit cutoff)  X (explicit cutoff) X (diameter for catastrophic collisions) will be neglected</t>
-  </si>
-  <si>
     <t xml:space="preserve">Seismic efficiency</t>
   </si>
   <si>
@@ -355,10 +379,34 @@
     <t xml:space="preserve">Ratio of Crater depth to Diameter</t>
   </si>
   <si>
-    <t xml:space="preserve">P wave speed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The P wave speed in the regolith as measured on the moon</t>
+    <t xml:space="preserve">Seismic Diffusivity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The diffusivity used in simulating seismic energy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bulk Modulus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The bulk modulus of grains at 1 Pa pressure</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shear Modulus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The shear modulus of the grains at 1 Pa pressure</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Failure wave</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P-wave</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P-wave, S-wave</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The dominant seismic energy wave</t>
   </si>
   <si>
     <t xml:space="preserve">Q</t>
@@ -367,10 +415,10 @@
     <t xml:space="preserve">Seismic quality factor</t>
   </si>
   <si>
-    <t xml:space="preserve">Frequency</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Seismic frequency</t>
+    <t xml:space="preserve">Beta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Momentum Enhancement efficiency factor</t>
   </si>
   <si>
     <t xml:space="preserve">Cummulative distribution</t>
@@ -480,7 +528,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -498,7 +546,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -507,6 +555,10 @@
     </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -518,7 +570,28 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <dxfs count="2">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF000000"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -715,7 +788,7 @@
         <v>11</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>4.3</v>
+        <v>4</v>
       </c>
       <c r="D5" s="3"/>
       <c r="E5" s="3" t="s">
@@ -745,7 +818,7 @@
         <v>11</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>0.01</v>
+        <v>2</v>
       </c>
       <c r="D7" s="3"/>
       <c r="E7" s="3" t="s">
@@ -893,43 +966,43 @@
         <v>38</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>39</v>
+        <v>11</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>50</v>
+        <v>15</v>
       </c>
       <c r="D3" s="3"/>
-      <c r="E3" s="3" t="s">
-        <v>40</v>
-      </c>
+      <c r="E3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>11</v>
+        <v>40</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>0.01</v>
+        <v>10</v>
       </c>
       <c r="D4" s="3"/>
       <c r="E4" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="B5" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" s="3" t="n">
-        <v>0.0001</v>
-      </c>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
     </row>
     <row r="6" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
@@ -939,7 +1012,7 @@
         <v>11</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>0.02</v>
+        <v>0.0001</v>
       </c>
       <c r="D6" s="3"/>
       <c r="E6" s="3"/>
@@ -949,185 +1022,215 @@
         <v>45</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>46</v>
+        <v>11</v>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>0.01</v>
       </c>
       <c r="D7" s="3"/>
-      <c r="E7" s="3" t="s">
-        <v>47</v>
-      </c>
+      <c r="E7" s="3"/>
     </row>
     <row r="8" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C8" s="3" t="n">
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>47</v>
       </c>
       <c r="D8" s="3"/>
       <c r="E8" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="B9" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="C9" s="3" t="n">
-        <v>1000</v>
-      </c>
-      <c r="D9" s="3"/>
+      <c r="D9" s="3" t="s">
+        <v>51</v>
+      </c>
       <c r="E9" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="C10" s="3" t="n">
-        <v>200</v>
-      </c>
-      <c r="D10" s="3"/>
+        <v>6</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>55</v>
+      </c>
       <c r="E10" s="3" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>39</v>
+        <v>11</v>
       </c>
       <c r="C11" s="3" t="n">
-        <v>200</v>
+        <v>0.05</v>
       </c>
       <c r="D11" s="3"/>
       <c r="E11" s="3" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>11</v>
+        <v>40</v>
       </c>
       <c r="C12" s="3" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="D12" s="3"/>
       <c r="E12" s="3" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>11</v>
+        <v>40</v>
       </c>
       <c r="C13" s="3" t="n">
-        <v>0.5</v>
+        <v>400</v>
       </c>
       <c r="D13" s="3"/>
       <c r="E13" s="3" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>30</v>
+        <v>40</v>
+      </c>
+      <c r="C14" s="3" t="n">
+        <v>400</v>
       </c>
       <c r="D14" s="3"/>
       <c r="E14" s="3" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>11</v>
       </c>
       <c r="C15" s="3" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="D15" s="3"/>
       <c r="E15" s="3" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C16" s="6" t="n">
-        <v>0.1</v>
+        <v>29</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>30</v>
       </c>
       <c r="D16" s="3"/>
       <c r="E16" s="3" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C17" s="6" t="n">
-        <v>1</v>
+      <c r="C17" s="3" t="n">
+        <v>10</v>
       </c>
       <c r="D17" s="3"/>
       <c r="E17" s="3" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="B18" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C18" s="6" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D18" s="3"/>
+      <c r="E18" s="3" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C19" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="3"/>
+      <c r="E19" s="3" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="B20" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C18" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="D18" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="E18" s="3" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+      <c r="C20" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>78</v>
+      </c>
+    </row>
     <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
@@ -1143,10 +1246,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
+  <sheetPr filterMode="true">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E1048576"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" zeroHeight="true" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20"/>
@@ -1176,7 +1279,7 @@
     </row>
     <row r="2" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>11</v>
@@ -1186,29 +1289,29 @@
       </c>
       <c r="D2" s="3"/>
       <c r="E2" s="3" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>6</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>11</v>
@@ -1218,12 +1321,12 @@
       </c>
       <c r="D4" s="3"/>
       <c r="E4" s="3" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>11</v>
@@ -1233,12 +1336,12 @@
       </c>
       <c r="D5" s="3"/>
       <c r="E5" s="3" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>11</v>
@@ -1248,12 +1351,12 @@
       </c>
       <c r="D6" s="3"/>
       <c r="E6" s="3" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>11</v>
@@ -1263,12 +1366,12 @@
       </c>
       <c r="D7" s="3"/>
       <c r="E7" s="3" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>11</v>
@@ -1278,43 +1381,69 @@
       </c>
       <c r="D8" s="3"/>
       <c r="E8" s="3" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>6</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="B10" s="3" t="s">
+      <c r="A10" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C10" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="D10" s="7"/>
+      <c r="E10" s="7" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="B11" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="C10" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="D10" s="3"/>
-      <c r="E10" s="3" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="1048576" customFormat="false" ht="60.4" hidden="true" customHeight="true" outlineLevel="0" collapsed="false"/>
+      <c r="C11" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="63.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="3"/>
+      <c r="B12" s="3"/>
+      <c r="C12" s="3"/>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
+    </row>
   </sheetData>
+  <autoFilter ref="A1048576">
+    <filterColumn colId="0" hiddenButton="1">
+      <filters blank="1"/>
+    </filterColumn>
+  </autoFilter>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -1322,6 +1451,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1330,7 +1460,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr defaultColWidth="10.1640625" defaultRowHeight="12.8" zeroHeight="true" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="17.83"/>
@@ -1360,7 +1490,7 @@
     </row>
     <row r="2" customFormat="false" ht="70.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>11</v>
@@ -1370,159 +1500,191 @@
       </c>
       <c r="D2" s="3"/>
       <c r="E2" s="3" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="70.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="62.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>97</v>
+        <v>106</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="3" t="n">
-        <v>0.1</v>
+      <c r="C3" s="6" t="n">
+        <v>1E-007</v>
       </c>
       <c r="D3" s="3"/>
       <c r="E3" s="3" t="s">
-        <v>98</v>
+        <v>107</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="62.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>11</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>1E-006</v>
+        <v>5500</v>
       </c>
       <c r="D4" s="3"/>
       <c r="E4" s="3" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="62.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>101</v>
+        <v>110</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" s="6" t="n">
-        <v>5500</v>
+        <v>6</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>111</v>
       </c>
       <c r="D5" s="3"/>
       <c r="E5" s="3" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="62.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="41.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>103</v>
+        <v>113</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>104</v>
+        <v>11</v>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>30</v>
       </c>
       <c r="D6" s="3"/>
       <c r="E6" s="3" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="41.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="50.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>11</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>30</v>
+        <v>0.2</v>
       </c>
       <c r="D7" s="3"/>
       <c r="E7" s="3" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="50.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="81.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>11</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>0.2</v>
+        <v>300</v>
       </c>
       <c r="D8" s="3"/>
       <c r="E8" s="3" t="s">
-        <v>109</v>
+        <v>118</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="81.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>110</v>
+        <v>119</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>11</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>100</v>
+        <v>96000</v>
       </c>
       <c r="D9" s="3"/>
       <c r="E9" s="3" t="s">
-        <v>111</v>
+        <v>120</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="81.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>112</v>
+        <v>121</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>11</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>1500</v>
+        <v>67000</v>
       </c>
       <c r="D10" s="3"/>
       <c r="E10" s="3" t="s">
-        <v>113</v>
+        <v>122</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="81.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C11" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D11" s="3"/>
+        <v>6</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>125</v>
+      </c>
       <c r="E11" s="3" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="71.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="81.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>116</v>
+        <v>127</v>
       </c>
       <c r="B12" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C12" s="6" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="81.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C13" s="6" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="71.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="B14" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>119</v>
+      <c r="C14" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>134</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated the functions and structure
</commit_message>
<xml_diff>
--- a/input/parameters.xlsx
+++ b/input/parameters.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="150">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -49,7 +49,7 @@
     <t xml:space="preserve">str</t>
   </si>
   <si>
-    <t xml:space="preserve">Bennu</t>
+    <t xml:space="preserve">Spherical</t>
   </si>
   <si>
     <t xml:space="preserve">Bennu, Ryugu, Itokawa, Spherical</t>
@@ -82,7 +82,7 @@
     <t xml:space="preserve">Output folder</t>
   </si>
   <si>
-    <t xml:space="preserve">Spherical_1</t>
+    <t xml:space="preserve">Debug</t>
   </si>
   <si>
     <t xml:space="preserve">The output folder of the simulations</t>
@@ -103,7 +103,7 @@
     <t xml:space="preserve">Dimension</t>
   </si>
   <si>
-    <t xml:space="preserve">2D</t>
+    <t xml:space="preserve">1D</t>
   </si>
   <si>
     <t xml:space="preserve">1D, 2D</t>
@@ -112,21 +112,36 @@
     <t xml:space="preserve">Dimension of simulation 1D or 2D</t>
   </si>
   <si>
+    <t xml:space="preserve">Single run</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bool</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No</t>
+  </si>
+  <si>
+    <t xml:space="preserve">To simulate a single landslide</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Visualization</t>
+  </si>
+  <si>
+    <t xml:space="preserve">If you want to do post processing of the already run simulation. Put the correct name in the output folder box.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Collision</t>
   </si>
   <si>
-    <t xml:space="preserve">bool</t>
+    <t xml:space="preserve">Do you want to include the effect of collision on spin rate?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Landslide</t>
   </si>
   <si>
     <t xml:space="preserve">Yes</t>
   </si>
   <si>
-    <t xml:space="preserve">Do you want to include the effect of collision on spin rate?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Landslide</t>
-  </si>
-  <si>
     <t xml:space="preserve">Do you want to include the effect of landslide on spin rate and shape?</t>
   </si>
   <si>
@@ -139,12 +154,27 @@
     <t xml:space="preserve">Static Friction angle</t>
   </si>
   <si>
-    <t xml:space="preserve">Friction angle of the regolith</t>
+    <t xml:space="preserve">Friction angle of the regolith used during the failure criteria</t>
   </si>
   <si>
     <t xml:space="preserve">Dynamic Friction angle</t>
   </si>
   <si>
+    <t xml:space="preserve">The friction angle used during the landslide motion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Failure profile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gaurav</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scheeres, Gaurav</t>
+  </si>
+  <si>
+    <t xml:space="preserve">File containing the functions to calculate the failure profile.</t>
+  </si>
+  <si>
     <t xml:space="preserve">dump</t>
   </si>
   <si>
@@ -163,9 +193,15 @@
     <t xml:space="preserve">Minimum epsilon</t>
   </si>
   <si>
+    <t xml:space="preserve">The minimum value of epsilon for which the code landslide model will run</t>
+  </si>
+  <si>
     <t xml:space="preserve">Maximum epsilon</t>
   </si>
   <si>
+    <t xml:space="preserve">The maximum value of epsilon that the landslide model will allow</t>
+  </si>
+  <si>
     <t xml:space="preserve">executable</t>
   </si>
   <si>
@@ -190,7 +226,7 @@
     <t xml:space="preserve">Reconstruction</t>
   </si>
   <si>
-    <t xml:space="preserve">Cartesian conserved variables</t>
+    <t xml:space="preserve">Primitive variables</t>
   </si>
   <si>
     <t xml:space="preserve">Primitive variables, Conserved variables, Cartesian conserved variables</t>
@@ -238,19 +274,31 @@
     <t xml:space="preserve">Maximum simulation period</t>
   </si>
   <si>
-    <t xml:space="preserve"> The simulation period after which the landslide will stop. This is the highest time for which landslide will be simulated</t>
+    <t xml:space="preserve"> The simulation period after which the landslide will stop. This is the highest time for which landslide will be simulated.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cohesion profile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exponential</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exponential, Linear, Constant </t>
+  </si>
+  <si>
+    <t xml:space="preserve">The profile of the cohesion with the depth.</t>
   </si>
   <si>
     <t xml:space="preserve">Cohesion constant</t>
   </si>
   <si>
-    <t xml:space="preserve"> Constant cohesion of the regolith</t>
+    <t xml:space="preserve"> Constant cohesion of the regolith.</t>
   </si>
   <si>
     <t xml:space="preserve">Cohesion linear</t>
   </si>
   <si>
-    <t xml:space="preserve">Linear increase in the cohesion with depth</t>
+    <t xml:space="preserve">Linear increase in the cohesion with depth.</t>
   </si>
   <si>
     <t xml:space="preserve">Friction type</t>
@@ -262,7 +310,7 @@
     <t xml:space="preserve">Constant, Variable</t>
   </si>
   <si>
-    <t xml:space="preserve">If you want a constant friction angle through out the lanslide, select constant otherwise choose variable</t>
+    <t xml:space="preserve">If you want a constant friction angle through out the lanslide, select constant otherwise choose variable.</t>
   </si>
   <si>
     <t xml:space="preserve">K</t>
@@ -332,9 +380,6 @@
   </si>
   <si>
     <t xml:space="preserve">stoc_yorp</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No</t>
   </si>
   <si>
     <t xml:space="preserve">Do you want yorp to be stochastic?</t>
@@ -705,7 +750,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" zeroHeight="true" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20"/>
@@ -788,7 +833,7 @@
         <v>11</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>4</v>
+        <v>3.15</v>
       </c>
       <c r="D5" s="3"/>
       <c r="E5" s="3" t="s">
@@ -818,7 +863,7 @@
         <v>11</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D7" s="3"/>
       <c r="E7" s="3" t="s">
@@ -901,6 +946,43 @@
       <c r="E12" s="3" t="s">
         <v>35</v>
       </c>
+    </row>
+    <row r="13" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="63.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="3"/>
+      <c r="B15" s="3"/>
+      <c r="C15" s="3"/>
+      <c r="D15" s="3"/>
+      <c r="E15" s="3"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -948,290 +1030,329 @@
     </row>
     <row r="2" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>11</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="D2" s="3"/>
       <c r="E2" s="3" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>11</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
+      <c r="E3" s="3" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="C4" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="D4" s="3"/>
+        <v>6</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>47</v>
+      </c>
       <c r="E4" s="3" t="s">
-        <v>41</v>
+        <v>48</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>11</v>
+        <v>50</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>0.01</v>
+        <v>50</v>
       </c>
       <c r="D5" s="3"/>
       <c r="E5" s="3" t="s">
-        <v>43</v>
+        <v>51</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>11</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>0.0001</v>
+        <v>0.01</v>
       </c>
       <c r="D6" s="3"/>
-      <c r="E6" s="3"/>
+      <c r="E6" s="3" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>45</v>
+        <v>54</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>11</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>0.01</v>
+        <v>0.0001</v>
       </c>
       <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
+      <c r="E7" s="3" t="s">
+        <v>55</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>46</v>
+        <v>56</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>47</v>
+        <v>11</v>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>0.01</v>
       </c>
       <c r="D8" s="3"/>
       <c r="E8" s="3" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>6</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>51</v>
-      </c>
+        <v>59</v>
+      </c>
+      <c r="D9" s="3"/>
       <c r="E9" s="3" t="s">
-        <v>52</v>
+        <v>60</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>6</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>56</v>
+        <v>64</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C11" s="3" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="D11" s="3"/>
+        <v>6</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>67</v>
+      </c>
       <c r="E11" s="3" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>59</v>
+        <v>69</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>40</v>
+        <v>11</v>
       </c>
       <c r="C12" s="3" t="n">
-        <v>1000</v>
+        <v>0.01</v>
       </c>
       <c r="D12" s="3"/>
       <c r="E12" s="3" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>61</v>
+        <v>71</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="C13" s="3" t="n">
-        <v>400</v>
+        <v>1000</v>
       </c>
       <c r="D13" s="3"/>
       <c r="E13" s="3" t="s">
-        <v>62</v>
+        <v>72</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>63</v>
+        <v>73</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="C14" s="3" t="n">
-        <v>400</v>
+        <v>200</v>
       </c>
       <c r="D14" s="3"/>
       <c r="E14" s="3" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>11</v>
+        <v>50</v>
       </c>
       <c r="C15" s="3" t="n">
-        <v>1</v>
+        <v>200</v>
       </c>
       <c r="D15" s="3"/>
       <c r="E15" s="3" t="s">
-        <v>66</v>
+        <v>76</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>67</v>
+        <v>77</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="C16" s="3" t="s">
-        <v>30</v>
+        <v>11</v>
+      </c>
+      <c r="C16" s="3" t="n">
+        <v>1</v>
       </c>
       <c r="D16" s="3"/>
       <c r="E16" s="3" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C17" s="3" t="n">
-        <v>10</v>
+        <v>29</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>37</v>
       </c>
       <c r="D17" s="3"/>
       <c r="E17" s="3" t="s">
-        <v>70</v>
+        <v>80</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C18" s="6" t="n">
-        <v>0.1</v>
+      <c r="C18" s="3" t="n">
+        <v>20</v>
       </c>
       <c r="D18" s="3"/>
       <c r="E18" s="3" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C19" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D19" s="3"/>
+        <v>6</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>85</v>
+      </c>
       <c r="E19" s="3" t="s">
-        <v>74</v>
+        <v>86</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>75</v>
+        <v>87</v>
       </c>
       <c r="B20" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C20" s="6" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D20" s="3"/>
+      <c r="E20" s="3" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C21" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" s="3"/>
+      <c r="E21" s="3" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="B22" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C20" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="D20" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="E20" s="3" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+      <c r="C22" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>94</v>
+      </c>
+    </row>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1279,7 +1400,7 @@
     </row>
     <row r="2" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>79</v>
+        <v>95</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>11</v>
@@ -1289,29 +1410,29 @@
       </c>
       <c r="D2" s="3"/>
       <c r="E2" s="3" t="s">
-        <v>80</v>
+        <v>96</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>81</v>
+        <v>97</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>6</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>82</v>
+        <v>98</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>83</v>
+        <v>99</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>84</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>85</v>
+        <v>101</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>11</v>
@@ -1321,12 +1442,12 @@
       </c>
       <c r="D4" s="3"/>
       <c r="E4" s="3" t="s">
-        <v>86</v>
+        <v>102</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>87</v>
+        <v>103</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>11</v>
@@ -1336,12 +1457,12 @@
       </c>
       <c r="D5" s="3"/>
       <c r="E5" s="3" t="s">
-        <v>88</v>
+        <v>104</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>89</v>
+        <v>105</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>11</v>
@@ -1351,12 +1472,12 @@
       </c>
       <c r="D6" s="3"/>
       <c r="E6" s="3" t="s">
-        <v>90</v>
+        <v>106</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>91</v>
+        <v>107</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>11</v>
@@ -1366,12 +1487,12 @@
       </c>
       <c r="D7" s="3"/>
       <c r="E7" s="3" t="s">
-        <v>92</v>
+        <v>108</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>93</v>
+        <v>109</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>11</v>
@@ -1381,29 +1502,29 @@
       </c>
       <c r="D8" s="3"/>
       <c r="E8" s="3" t="s">
-        <v>94</v>
+        <v>110</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>95</v>
+        <v>111</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>6</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>96</v>
+        <v>112</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>97</v>
+        <v>113</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>98</v>
+        <v>114</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="B10" s="7" t="s">
         <v>11</v>
@@ -1413,22 +1534,22 @@
       </c>
       <c r="D10" s="7"/>
       <c r="E10" s="7" t="s">
-        <v>100</v>
+        <v>116</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="63.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>101</v>
+        <v>117</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>29</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>102</v>
+        <v>30</v>
       </c>
       <c r="D11" s="3"/>
       <c r="E11" s="3" t="s">
-        <v>103</v>
+        <v>118</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="63.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1490,7 +1611,7 @@
     </row>
     <row r="2" customFormat="false" ht="70.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>104</v>
+        <v>119</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>11</v>
@@ -1500,27 +1621,27 @@
       </c>
       <c r="D2" s="3"/>
       <c r="E2" s="3" t="s">
-        <v>105</v>
+        <v>120</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="62.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>106</v>
+        <v>121</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>11</v>
       </c>
       <c r="C3" s="6" t="n">
-        <v>1E-007</v>
+        <v>3E-007</v>
       </c>
       <c r="D3" s="3"/>
       <c r="E3" s="3" t="s">
-        <v>107</v>
+        <v>122</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="62.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>108</v>
+        <v>123</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>11</v>
@@ -1530,27 +1651,27 @@
       </c>
       <c r="D4" s="3"/>
       <c r="E4" s="3" t="s">
-        <v>109</v>
+        <v>124</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="62.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>110</v>
+        <v>125</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>6</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>111</v>
+        <v>126</v>
       </c>
       <c r="D5" s="3"/>
       <c r="E5" s="3" t="s">
-        <v>112</v>
+        <v>127</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="41.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>113</v>
+        <v>128</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>11</v>
@@ -1560,12 +1681,12 @@
       </c>
       <c r="D6" s="3"/>
       <c r="E6" s="3" t="s">
-        <v>114</v>
+        <v>129</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="50.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>115</v>
+        <v>130</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>11</v>
@@ -1575,12 +1696,12 @@
       </c>
       <c r="D7" s="3"/>
       <c r="E7" s="3" t="s">
-        <v>116</v>
+        <v>131</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="81.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>117</v>
+        <v>132</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>11</v>
@@ -1590,12 +1711,12 @@
       </c>
       <c r="D8" s="3"/>
       <c r="E8" s="3" t="s">
-        <v>118</v>
+        <v>133</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="81.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>119</v>
+        <v>134</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>11</v>
@@ -1605,12 +1726,12 @@
       </c>
       <c r="D9" s="3"/>
       <c r="E9" s="3" t="s">
-        <v>120</v>
+        <v>135</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="81.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>121</v>
+        <v>136</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>11</v>
@@ -1620,29 +1741,29 @@
       </c>
       <c r="D10" s="3"/>
       <c r="E10" s="3" t="s">
-        <v>122</v>
+        <v>137</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="81.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>123</v>
+        <v>138</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>6</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>124</v>
+        <v>139</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>125</v>
+        <v>140</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>126</v>
+        <v>141</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="81.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>127</v>
+        <v>142</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>11</v>
@@ -1652,12 +1773,12 @@
       </c>
       <c r="D12" s="3"/>
       <c r="E12" s="3" t="s">
-        <v>128</v>
+        <v>143</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="81.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>129</v>
+        <v>144</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>11</v>
@@ -1667,24 +1788,24 @@
       </c>
       <c r="D13" s="3"/>
       <c r="E13" s="3" t="s">
-        <v>130</v>
+        <v>145</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="71.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>131</v>
+        <v>146</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>6</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>132</v>
+        <v>147</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>133</v>
+        <v>148</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>134</v>
+        <v>149</v>
       </c>
     </row>
   </sheetData>

</xml_diff>